<commit_message>
chore: update component list
</commit_message>
<xml_diff>
--- a/새싹_부품_리스트.xlsx
+++ b/새싹_부품_리스트.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t xml:space="preserve">BUDGET: </t>
   </si>
@@ -240,6 +240,54 @@
   <si>
     <t>https://www.coupang.com/vp/products/8427726478</t>
   </si>
+  <si>
+    <t>https://www.devicemart.co.kr/goods/view?no=15267411</t>
+  </si>
+  <si>
+    <t>[SMG] SN65HVD23x 5V CAN통신 트랜시버 [TYE-CT003]</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/epep3724/products/13318666874?is_retargeting=true&amp;c=260101_p_Naver_product&amp;pid=Naver&amp;deep_link_value=https%3A%2F%2Fsmartstore.naver.com%2Fepep3724%2Fproducts%2F13318666874%3Fka_ref%3Dkakao%26ka_req_id%3DgH3XYBfDIohsLlXI9dF8AA%26ka_template%3Dcommerce_basic&amp;dtm_source=KK&amp;dtm_detail=gH3XYBfDIohsLlXI9dF8AA&amp;dtm_campaign=commerce_basic&amp;dtm_medium=OG</t>
+  </si>
+  <si>
+    <t>https://smartstore.naver.com/epep3724/products/13318666874</t>
+  </si>
+  <si>
+    <t>인코더 모터 12V</t>
+  </si>
+  <si>
+    <t>1590RPM</t>
+  </si>
+  <si>
+    <t>옵션 1590RPM</t>
+  </si>
+  <si>
+    <t>모터쉴드</t>
+  </si>
+  <si>
+    <t>https://www.devicemart.co.kr/goods/view?no=15960220</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Voltly] MCP2515 CAN BUS TJA1050 수신기 [VLT-CAN001] </t>
+  </si>
+  <si>
+    <t>https://roboroboshop.com/product/%ED%94%84%EB%A0%88%EC%9E%84-big-mainpcb/77/category/177/display/1/#prdInfo</t>
+  </si>
+  <si>
+    <t>배송비 3500원 포함</t>
+  </si>
+  <si>
+    <t>프레임 - Big Main[PCB]</t>
+  </si>
+  <si>
+    <t>https://www.devicemart.co.kr/goods/view?no=3164</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> [아세아볼트] PCB서포트용 나사(니켈) M3X5 </t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
 </sst>
 </file>
 
@@ -248,7 +296,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="[$₩]#,##0"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="35">
     <font>
       <sz val="10.0"/>
       <name val="Arial"/>
@@ -463,14 +511,8 @@
       <scheme val="minor"/>
       <color rgb="FF7F7F7F"/>
     </font>
-    <font>
-      <u/>
-      <sz val="10.0"/>
-      <name val="맑은 고딕"/>
-      <color theme="10"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -669,6 +711,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399980"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -865,7 +919,6 @@
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
@@ -874,7 +927,6 @@
       <bottom style="thick">
         <color theme="4"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
@@ -883,7 +935,6 @@
       <bottom style="thick">
         <color rgb="FFACCCEA"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
@@ -892,7 +943,6 @@
       <bottom style="medium">
         <color theme="4" tint="0.399980"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -907,7 +957,6 @@
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -922,7 +971,6 @@
       <bottom style="thin">
         <color rgb="FF3F3F3F"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="double">
@@ -937,7 +985,6 @@
       <bottom style="double">
         <color rgb="FF3F3F3F"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
@@ -946,7 +993,6 @@
       <bottom style="double">
         <color rgb="FFFF8001"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
@@ -957,7 +1003,6 @@
       <bottom style="double">
         <color theme="4"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
@@ -1109,7 +1154,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1216,7 +1261,77 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="34" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="34" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="34" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="35" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="35" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="35" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="35" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="35" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="35" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="35" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="20% - Accent1" xfId="25" builtinId="30"/>
@@ -1470,13 +1585,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultColWidth="12.66406250" defaultRowHeight="15.750000" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.71928583" customWidth="1" outlineLevel="0"/>
     <col min="2" max="2" width="7.71928583" customWidth="1" outlineLevel="0"/>
     <col min="3" max="3" width="5.86214290" customWidth="1" outlineLevel="0"/>
-    <col min="4" max="4" width="36.14785658" customWidth="1" outlineLevel="0"/>
+    <col min="4" max="4" width="54.71928678" customWidth="1" outlineLevel="0"/>
     <col min="5" max="5" width="8.29071413" customWidth="1" outlineLevel="0"/>
     <col min="6" max="7" width="14.14785753" customWidth="1" outlineLevel="0"/>
     <col min="8" max="8" style="13" width="14.14785753" customWidth="1" outlineLevel="0"/>
@@ -1553,7 +1668,7 @@
       </c>
       <c r="G5" s="27">
         <f>1000000-G33</f>
-        <v>251900</v>
+        <v>11310</v>
       </c>
       <c r="H5" s="11"/>
       <c r="I5" s="5"/>
@@ -1617,35 +1732,35 @@
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="15.000000">
-      <c r="A8" s="6"/>
-      <c r="B8" s="19">
+    <row r="8" spans="1:11" s="60" customFormat="1" ht="15.000000">
+      <c r="A8" s="62"/>
+      <c r="B8" s="63">
         <v>2</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="29"/>
-      <c r="E8" s="22">
+      <c r="D8" s="65"/>
+      <c r="E8" s="66">
         <v>1</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="67">
         <v>110650</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="67">
         <f>E8*F8</f>
         <v>110650</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="I8" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="31" t="s">
+      <c r="J8" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="K8" s="7"/>
+      <c r="K8" s="70"/>
     </row>
     <row r="9" spans="1:11" ht="15.000000">
       <c r="A9" s="6"/>
@@ -1674,35 +1789,35 @@
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="15.000000">
-      <c r="A10" s="6"/>
-      <c r="B10" s="19">
+    <row r="10" spans="1:11" s="60" customFormat="1" ht="15.000000">
+      <c r="A10" s="62"/>
+      <c r="B10" s="63">
         <v>4</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="29"/>
-      <c r="E10" s="22">
+      <c r="D10" s="65"/>
+      <c r="E10" s="66">
         <v>3</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="67">
         <v>5450</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="67">
         <f>E10*F10+3000</f>
         <v>19350</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="21" t="s">
+      <c r="I10" s="68" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="33" t="s">
+      <c r="J10" s="69" t="s">
         <v>46</v>
       </c>
-      <c r="K10" s="7"/>
+      <c r="K10" s="70"/>
     </row>
     <row r="11" spans="1:11" ht="15.000000">
       <c r="A11" s="6"/>
@@ -1766,7 +1881,7 @@
     </row>
     <row r="13" spans="1:11" ht="15.000000">
       <c r="A13" s="6"/>
-      <c r="B13" s="19">
+      <c r="B13" s="63">
         <v>7</v>
       </c>
       <c r="C13" s="28" t="s">
@@ -2005,7 +2120,7 @@
       </c>
       <c r="K20" s="7"/>
     </row>
-    <row r="21" spans="1:16" ht="15.000000">
+    <row r="21" spans="1:16">
       <c r="A21" s="6"/>
       <c r="B21" s="19">
         <v>15</v>
@@ -2118,14 +2233,14 @@
         <v>12</v>
       </c>
       <c r="I24" s="21"/>
-      <c r="J24" s="48" t="s">
+      <c r="J24" s="33" t="s">
         <v>66</v>
       </c>
       <c r="K24" s="7"/>
     </row>
     <row r="25" spans="1:16" ht="15.000000">
       <c r="A25" s="6"/>
-      <c r="B25" s="19">
+      <c r="B25" s="63">
         <v>19</v>
       </c>
       <c r="C25" s="28" t="s">
@@ -2185,93 +2300,153 @@
     </row>
     <row r="27" spans="1:16" ht="15.000000">
       <c r="A27" s="6"/>
-      <c r="B27" s="19">
+      <c r="B27" s="63">
         <v>21</v>
       </c>
-      <c r="C27" s="28"/>
+      <c r="C27" s="28" t="s">
+        <v>68</v>
+      </c>
       <c r="D27" s="29"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="20"/>
+      <c r="E27" s="22">
+        <v>1</v>
+      </c>
+      <c r="F27" s="20">
+        <v>13200</v>
+      </c>
       <c r="G27" s="20">
         <f>E27*F27</f>
-        <v>0</v>
-      </c>
-      <c r="H27" s="19"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="33"/>
+        <v>13200</v>
+      </c>
+      <c r="H27" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I27" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="J27" s="33" t="s">
+        <v>67</v>
+      </c>
       <c r="K27" s="7"/>
     </row>
     <row r="28" spans="1:16" ht="15.000000">
       <c r="A28" s="6"/>
-      <c r="B28" s="19">
+      <c r="B28" s="75">
         <v>22</v>
       </c>
-      <c r="C28" s="28"/>
+      <c r="C28" s="28" t="s">
+        <v>71</v>
+      </c>
       <c r="D28" s="29"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="20"/>
+      <c r="E28" s="22">
+        <v>4</v>
+      </c>
+      <c r="F28" s="20">
+        <v>48020</v>
+      </c>
       <c r="G28" s="20">
         <f>E28*F28</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="19"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="31"/>
+        <v>192080</v>
+      </c>
+      <c r="H28" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="I28" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="J28" s="31" t="s">
+        <v>70</v>
+      </c>
       <c r="K28" s="7"/>
     </row>
-    <row r="29" spans="1:16" ht="15.000000">
-      <c r="A29" s="6"/>
-      <c r="B29" s="19">
+    <row r="29" spans="1:16" s="60" customFormat="1" ht="13.500000">
+      <c r="A29" s="62"/>
+      <c r="B29" s="63">
         <v>23</v>
       </c>
-      <c r="C29" s="28"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="20">
+      <c r="C29" s="64" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" s="65"/>
+      <c r="E29" s="66">
+        <v>3</v>
+      </c>
+      <c r="F29" s="67">
+        <v>1870</v>
+      </c>
+      <c r="G29" s="67">
         <f>E29*F29</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="19"/>
-      <c r="I29" s="21"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="7"/>
-    </row>
-    <row r="30" spans="1:16" ht="15.000000">
-      <c r="A30" s="6"/>
-      <c r="B30" s="19">
+        <v>5610</v>
+      </c>
+      <c r="H29" s="63" t="s">
+        <v>7</v>
+      </c>
+      <c r="I29" s="68" t="s">
+        <v>18</v>
+      </c>
+      <c r="J29" s="69" t="s">
+        <v>75</v>
+      </c>
+      <c r="K29" s="70"/>
+    </row>
+    <row r="30" spans="1:16" s="60" customFormat="1" ht="15.000000">
+      <c r="A30" s="62"/>
+      <c r="B30" s="63">
         <v>24</v>
       </c>
-      <c r="C30" s="28"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20">
-        <f>E30*F30</f>
-        <v>0</v>
-      </c>
-      <c r="H30" s="19"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="33"/>
-      <c r="K30" s="7"/>
-    </row>
-    <row r="31" spans="1:16" ht="15.000000">
-      <c r="A31" s="6"/>
-      <c r="B31" s="19">
+      <c r="C30" s="64" t="s">
+        <v>79</v>
+      </c>
+      <c r="D30" s="65"/>
+      <c r="E30" s="66">
+        <v>3</v>
+      </c>
+      <c r="F30" s="67">
+        <v>8000</v>
+      </c>
+      <c r="G30" s="67">
+        <f>E30*F30+3500</f>
+        <v>27500</v>
+      </c>
+      <c r="H30" s="63" t="s">
+        <v>13</v>
+      </c>
+      <c r="I30" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="J30" s="69" t="s">
+        <v>77</v>
+      </c>
+      <c r="K30" s="70"/>
+    </row>
+    <row r="31" spans="1:16" s="60" customFormat="1" ht="13.500000">
+      <c r="A31" s="62"/>
+      <c r="B31" s="63">
         <v>25</v>
       </c>
-      <c r="C31" s="28"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20">
+      <c r="C31" s="64" t="s">
+        <v>81</v>
+      </c>
+      <c r="D31" s="65"/>
+      <c r="E31" s="66">
+        <v>200</v>
+      </c>
+      <c r="F31" s="67">
+        <v>11</v>
+      </c>
+      <c r="G31" s="67">
         <f>E31*F31</f>
-        <v>0</v>
-      </c>
-      <c r="H31" s="19"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="21"/>
-      <c r="K31" s="7"/>
+        <v>2200</v>
+      </c>
+      <c r="H31" s="63" t="s">
+        <v>7</v>
+      </c>
+      <c r="I31" s="68" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="69" t="s">
+        <v>80</v>
+      </c>
+      <c r="K31" s="70"/>
     </row>
     <row r="32" spans="1:16" ht="15.000000">
       <c r="A32" s="6"/>
@@ -2304,7 +2479,7 @@
       </c>
       <c r="G33" s="15">
         <f>SUM(G7:G32)</f>
-        <v>748100</v>
+        <v>988690</v>
       </c>
       <c r="H33" s="16"/>
       <c r="I33" s="17"/>
@@ -2355,6 +2530,11 @@
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
+    </row>
+    <row r="37" spans="1:11">
+      <c r="C37" s="0" t="s">
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="32">
@@ -2393,7 +2573,7 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H30 H7:H28">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H7:H26 H27 H28 H29 H30 H31">
       <formula1>"디바이스마트,쿠팡,기타"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2410,6 +2590,9 @@
     <hyperlink r:id="rId10" ref="J17"/>
     <hyperlink r:id="rId11" ref="J19"/>
     <hyperlink r:id="rId12" ref="J24"/>
+    <hyperlink r:id="rId13" ref="J29"/>
+    <hyperlink r:id="rId14" ref="J21"/>
+    <hyperlink r:id="rId15" ref="J31"/>
   </hyperlinks>
   <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
   <pageSetup paperSize="9" scale="59" fitToWidth="0" fitToHeight="0" orientation="portrait"/>

</xml_diff>

<commit_message>
fix(reqs): SYS025/SWR012 를 DBC(6byte, 20/10ms) 에 정합 + 토폴로지 문구 유지
stash pop 충돌 해결. ACC-CANDB/acc_db.dbc 를 ground truth 로 삼아 병합:

- SYS025: HB 주기를 500ms → 20/10/10ms (DBC GenMsgCycleTime 과 일치),
  타임아웃 60/30/30ms 명시, ECU HB 에 ASIL-B per SAF018 표기 유지,
  MTR HB 가 CAN 게이트웨이 Arduino 송신임을 나타내는 I2C 중계 노트 유지.
- SWR012: DLC 8 → 6 bytes (PWM 4ch + MTR_RC 4bit + MTR_CRC 8bit,
  E2E P01 per SAF010 ASIL-B) 로 수정. 4휠 DBC 복제 / Arduino 게이트웨이
  I2C 중계 / 대표 바퀴 1개 구동 설명은 유지.
- SAF010: MTR_CMD 0x210 + DLC 6 byte + MTR_RC/MTR_CRC 로 갱신 (auto-merge).
- strictdoc_config.py: exclude_doc_paths 에 .venv 추가.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/새싹_부품_리스트.xlsx
+++ b/새싹_부품_리스트.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Polaris Office MAC Sheet" lastEdited="7" lowestEdited="7" rupBuild=""/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\acc\ACC-docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078AD98A-AFCF-4C3E-9AD3-C43F3B266EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시트1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="79">
   <si>
     <t xml:space="preserve">BUDGET: </t>
   </si>
@@ -94,6 +99,8 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Malgun Gothic"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>개포동</t>
     </r>
@@ -102,6 +109,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -110,6 +118,8 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Malgun Gothic"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>잡초</t>
     </r>
@@ -214,9 +224,6 @@
     <t>라즈베리파이 카메라 브라켓</t>
   </si>
   <si>
-    <t>https://www.coupang.com/vp/products/8427726478?itemId=24379351616&amp;searchId=feed-f1abfe00352148358e5f66b9bdd5c89f-3.3.37%3Aview_together_ads-P6211119595&amp;vendorItemId=91394465314&amp;sourceType=SDP_ADS&amp;clickEventId=c5698ff0-299d-11f1-a5a4-ecab0275ebfb</t>
-  </si>
-  <si>
     <t>양면테이프</t>
   </si>
   <si>
@@ -247,18 +254,12 @@
     <t>[SMG] SN65HVD23x 5V CAN통신 트랜시버 [TYE-CT003]</t>
   </si>
   <si>
-    <t>https://smartstore.naver.com/epep3724/products/13318666874?is_retargeting=true&amp;c=260101_p_Naver_product&amp;pid=Naver&amp;deep_link_value=https%3A%2F%2Fsmartstore.naver.com%2Fepep3724%2Fproducts%2F13318666874%3Fka_ref%3Dkakao%26ka_req_id%3DgH3XYBfDIohsLlXI9dF8AA%26ka_template%3Dcommerce_basic&amp;dtm_source=KK&amp;dtm_detail=gH3XYBfDIohsLlXI9dF8AA&amp;dtm_campaign=commerce_basic&amp;dtm_medium=OG</t>
-  </si>
-  <si>
     <t>https://smartstore.naver.com/epep3724/products/13318666874</t>
   </si>
   <si>
     <t>인코더 모터 12V</t>
   </si>
   <si>
-    <t>1590RPM</t>
-  </si>
-  <si>
     <t>옵션 1590RPM</t>
   </si>
   <si>
@@ -284,243 +285,150 @@
   </si>
   <si>
     <t xml:space="preserve"> [아세아볼트] PCB서포트용 나사(니켈) M3X5 </t>
-  </si>
-  <si>
-    <t>a</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="[$₩]#,##0"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="18">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-      <color rgb="FF000000"/>
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Noto Sans SC"/>
-      <color theme="1"/>
     </font>
     <font>
       <i/>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color rgb="FFD9D9D9"/>
       <name val="Noto Sans SC"/>
-      <color rgb="FFD9D9D9"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Noto Sans SC"/>
-      <color theme="1"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
-      <color theme="1"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <color rgb="FF000000"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="10"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
-      <color theme="10"/>
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
-      <color theme="1"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="FF000000"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="맑은 고딕"/>
-      <color theme="1"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="맑은 고딕"/>
-      <color theme="1"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="FF000000"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color rgb="FFB7B7B7"/>
       <name val="맑은 고딕"/>
-      <color rgb="FFB7B7B7"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="맑은 고딕"/>
-      <color theme="1"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="5"/>
       <name val="맑은 고딕"/>
-      <color theme="5"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Malgun Gothic"/>
-      <color rgb="FF000000"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
+      <color theme="11"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
-      <color theme="11"/>
     </font>
     <font>
       <u/>
-      <sz val="10.0"/>
+      <sz val="10"/>
+      <color theme="10"/>
       <name val="맑은 고딕"/>
-      <color theme="10"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FFFF0000"/>
-    </font>
-    <font>
-      <sz val="18.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color theme="3"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color theme="3"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color theme="3"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color theme="3"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FF3F3F76"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FF3F3F3F"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FFFA7D00"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FFFA7D00"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color theme="1"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FF006100"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FF9C0006"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FF9C6500"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color theme="0"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color theme="1"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11.0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-      <color rgb="FF7F7F7F"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -530,209 +438,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599990"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599990"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599990"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599990"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599990"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599990"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399980"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="16">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -747,6 +464,7 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -759,6 +477,7 @@
         <color rgb="FFFFFFFF"/>
       </top>
       <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -771,6 +490,7 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -785,6 +505,7 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -797,6 +518,7 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -809,6 +531,7 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -821,6 +544,7 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -831,6 +555,7 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -839,6 +564,7 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -849,6 +575,7 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -861,6 +588,7 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -873,6 +601,7 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -883,6 +612,7 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -895,6 +625,7 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -905,485 +636,155 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color rgb="FFACCCEA"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.399980"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="7" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="5" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyFont="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" applyAlignment="0" applyFont="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="20" applyAlignment="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="21" applyAlignment="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="20" applyAlignment="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="22" applyAlignment="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="23" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="24" applyAlignment="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="11" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="15" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="16" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="19" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="24" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="27" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="176" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="176" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="34" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="34" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="34" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="34" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="35" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="35" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="35" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="35" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="20% - Accent1" xfId="25" builtinId="30"/>
-    <cellStyle name="20% - Accent2" xfId="29" builtinId="34"/>
-    <cellStyle name="20% - Accent3" xfId="33" builtinId="38"/>
-    <cellStyle name="20% - Accent4" xfId="37" builtinId="42"/>
-    <cellStyle name="20% - Accent5" xfId="41" builtinId="46"/>
-    <cellStyle name="20% - Accent6" xfId="45" builtinId="50"/>
-    <cellStyle name="40% - Accent1" xfId="26" builtinId="31"/>
-    <cellStyle name="40% - Accent2" xfId="30" builtinId="35"/>
-    <cellStyle name="40% - Accent3" xfId="34" builtinId="39"/>
-    <cellStyle name="40% - Accent4" xfId="38" builtinId="43"/>
-    <cellStyle name="40% - Accent5" xfId="42" builtinId="47"/>
-    <cellStyle name="40% - Accent6" xfId="46" builtinId="51"/>
-    <cellStyle name="60% - Accent1" xfId="27" builtinId="32"/>
-    <cellStyle name="60% - Accent2" xfId="31" builtinId="36"/>
-    <cellStyle name="60% - Accent3" xfId="35" builtinId="40"/>
-    <cellStyle name="60% - Accent4" xfId="39" builtinId="44"/>
-    <cellStyle name="60% - Accent5" xfId="43" builtinId="48"/>
-    <cellStyle name="60% - Accent6" xfId="47" builtinId="52"/>
-    <cellStyle name="Accent1" xfId="24" builtinId="29"/>
-    <cellStyle name="Accent2" xfId="28" builtinId="33"/>
-    <cellStyle name="Accent3" xfId="32" builtinId="37"/>
-    <cellStyle name="Accent4" xfId="36" builtinId="41"/>
-    <cellStyle name="Accent5" xfId="40" builtinId="45"/>
-    <cellStyle name="Accent6" xfId="44" builtinId="49"/>
-    <cellStyle name="Bad" xfId="22" builtinId="27"/>
-    <cellStyle name="Calculation" xfId="17" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="18" builtinId="23"/>
-    <cellStyle name="Comma" xfId="3" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="6" builtinId="6"/>
-    <cellStyle name="Currency" xfId="4" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="7" builtinId="7"/>
-    <cellStyle name="Explanatory Text" xfId="48" builtinId="53"/>
-    <cellStyle name="Good" xfId="21" builtinId="26"/>
-    <cellStyle name="Heading 1" xfId="11" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="12" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="13" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="14" builtinId="19"/>
-    <cellStyle name="Input" xfId="15" builtinId="20"/>
-    <cellStyle name="Linked Cell" xfId="19" builtinId="24"/>
-    <cellStyle name="Neutral" xfId="23" builtinId="28"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Output" xfId="16" builtinId="21"/>
-    <cellStyle name="Percent" xfId="5" builtinId="5"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Total" xfId="20" builtinId="25"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+  <cellStyles count="3">
     <cellStyle name="열어 본 하이퍼링크" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
     <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1584,23 +985,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P37"/>
-  <sheetFormatPr defaultColWidth="12.66406250" defaultRowHeight="15.750000" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="5.71928583" customWidth="1" outlineLevel="0"/>
-    <col min="2" max="2" width="7.71928583" customWidth="1" outlineLevel="0"/>
-    <col min="3" max="3" width="5.86214290" customWidth="1" outlineLevel="0"/>
-    <col min="4" max="4" width="54.71928678" customWidth="1" outlineLevel="0"/>
-    <col min="5" max="5" width="8.29071413" customWidth="1" outlineLevel="0"/>
-    <col min="6" max="7" width="14.14785753" customWidth="1" outlineLevel="0"/>
-    <col min="8" max="8" style="13" width="14.14785753" customWidth="1" outlineLevel="0"/>
-    <col min="9" max="9" width="27.00499998" customWidth="1" outlineLevel="0"/>
-    <col min="10" max="10" width="59.86214338" customWidth="1" outlineLevel="0"/>
-    <col min="11" max="11" width="8.86214243" customWidth="1" outlineLevel="0"/>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" customWidth="1"/>
+    <col min="3" max="3" width="5.85546875" customWidth="1"/>
+    <col min="4" max="4" width="54.7109375" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" customWidth="1"/>
+    <col min="6" max="7" width="14.140625" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" style="13" customWidth="1"/>
+    <col min="9" max="9" width="27" customWidth="1"/>
+    <col min="10" max="10" width="59.85546875" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.000000">
+    <row r="1" spans="1:11" ht="12.75">
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
@@ -1612,14 +1013,14 @@
       <c r="J1" s="8"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="17.000000">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="2"/>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="36"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="38"/>
       <c r="F2" s="23"/>
       <c r="G2" s="23"/>
       <c r="H2" s="9"/>
@@ -1627,7 +1028,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" ht="12.450000" customHeight="1">
+    <row r="3" spans="1:11" ht="12.4" customHeight="1">
       <c r="A3" s="3"/>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
@@ -1640,12 +1041,12 @@
       <c r="J3" s="4"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" ht="16.750000" customHeight="1">
+    <row r="4" spans="1:11" ht="16.7" customHeight="1">
       <c r="A4" s="3"/>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="38"/>
+      <c r="C4" s="40"/>
       <c r="D4" s="30" t="s">
         <v>24</v>
       </c>
@@ -1655,14 +1056,14 @@
       <c r="J4" s="4"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" ht="22.750000" customHeight="1">
+    <row r="5" spans="1:11" ht="22.7" customHeight="1">
       <c r="A5" s="3"/>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="41"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="43"/>
       <c r="F5" s="26" t="s">
         <v>0</v>
       </c>
@@ -1675,15 +1076,15 @@
       <c r="J5" s="5"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" ht="15.000000">
+    <row r="6" spans="1:11" ht="13.5">
       <c r="A6" s="6"/>
       <c r="B6" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="43"/>
+      <c r="D6" s="45"/>
       <c r="E6" s="18" t="s">
         <v>3</v>
       </c>
@@ -1704,15 +1105,15 @@
       </c>
       <c r="K6" s="7"/>
     </row>
-    <row r="7" spans="1:11" ht="15.000000">
+    <row r="7" spans="1:11" ht="13.5">
       <c r="A7" s="6"/>
       <c r="B7" s="19">
         <v>1</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="29"/>
+      <c r="D7" s="47"/>
       <c r="E7" s="22">
         <v>1</v>
       </c>
@@ -1732,45 +1133,45 @@
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" s="60" customFormat="1" ht="15.000000">
-      <c r="A8" s="62"/>
-      <c r="B8" s="63">
+    <row r="8" spans="1:11" ht="13.5">
+      <c r="A8" s="6"/>
+      <c r="B8" s="19">
         <v>2</v>
       </c>
-      <c r="C8" s="64" t="s">
+      <c r="C8" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="65"/>
-      <c r="E8" s="66">
+      <c r="D8" s="47"/>
+      <c r="E8" s="22">
         <v>1</v>
       </c>
-      <c r="F8" s="67">
+      <c r="F8" s="20">
         <v>110650</v>
       </c>
-      <c r="G8" s="67">
+      <c r="G8" s="20">
         <f>E8*F8</f>
         <v>110650</v>
       </c>
-      <c r="H8" s="63" t="s">
+      <c r="H8" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="68" t="s">
+      <c r="I8" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="71" t="s">
+      <c r="J8" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="K8" s="70"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.000000">
+      <c r="K8" s="7"/>
+    </row>
+    <row r="9" spans="1:11" ht="13.5">
       <c r="A9" s="6"/>
       <c r="B9" s="19">
         <v>3</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="29"/>
+      <c r="D9" s="47"/>
       <c r="E9" s="22">
         <v>1</v>
       </c>
@@ -1789,45 +1190,45 @@
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" s="60" customFormat="1" ht="15.000000">
-      <c r="A10" s="62"/>
-      <c r="B10" s="63">
+    <row r="10" spans="1:11" ht="13.5">
+      <c r="A10" s="6"/>
+      <c r="B10" s="19">
         <v>4</v>
       </c>
-      <c r="C10" s="64" t="s">
+      <c r="C10" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="65"/>
-      <c r="E10" s="66">
+      <c r="D10" s="47"/>
+      <c r="E10" s="22">
         <v>3</v>
       </c>
-      <c r="F10" s="67">
+      <c r="F10" s="20">
         <v>5450</v>
       </c>
-      <c r="G10" s="67">
+      <c r="G10" s="20">
         <f>E10*F10+3000</f>
         <v>19350</v>
       </c>
-      <c r="H10" s="63" t="s">
+      <c r="H10" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="68" t="s">
+      <c r="I10" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="69" t="s">
+      <c r="J10" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="K10" s="70"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.000000">
+      <c r="K10" s="7"/>
+    </row>
+    <row r="11" spans="1:11" ht="13.5">
       <c r="A11" s="6"/>
       <c r="B11" s="19">
         <v>5</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="29"/>
+      <c r="D11" s="47"/>
       <c r="E11" s="22">
         <v>2</v>
       </c>
@@ -1835,7 +1236,7 @@
         <v>9900</v>
       </c>
       <c r="G11" s="20">
-        <f>E11*F11</f>
+        <f t="shared" ref="G11:G22" si="0">E11*F11</f>
         <v>19800</v>
       </c>
       <c r="H11" s="19" t="s">
@@ -1849,15 +1250,15 @@
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="15.000000">
+    <row r="12" spans="1:11" ht="13.5">
       <c r="A12" s="6"/>
       <c r="B12" s="19">
         <v>6</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="29"/>
+      <c r="D12" s="47"/>
       <c r="E12" s="22">
         <v>1</v>
       </c>
@@ -1865,7 +1266,7 @@
         <v>116600</v>
       </c>
       <c r="G12" s="20">
-        <f>E12*F12</f>
+        <f t="shared" si="0"/>
         <v>116600</v>
       </c>
       <c r="H12" s="19" t="s">
@@ -1879,15 +1280,15 @@
       </c>
       <c r="K12" s="7"/>
     </row>
-    <row r="13" spans="1:11" ht="15.000000">
+    <row r="13" spans="1:11" ht="13.5">
       <c r="A13" s="6"/>
-      <c r="B13" s="63">
+      <c r="B13" s="19">
         <v>7</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="29"/>
+      <c r="D13" s="47"/>
       <c r="E13" s="22">
         <v>1</v>
       </c>
@@ -1895,7 +1296,7 @@
         <v>65000</v>
       </c>
       <c r="G13" s="20">
-        <f>E13*F13</f>
+        <f t="shared" si="0"/>
         <v>65000</v>
       </c>
       <c r="H13" s="19" t="s">
@@ -1909,15 +1310,15 @@
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="15.000000">
+    <row r="14" spans="1:11" ht="13.5">
       <c r="A14" s="6"/>
       <c r="B14" s="19">
         <v>8</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="29"/>
+      <c r="D14" s="47"/>
       <c r="E14" s="22">
         <v>2</v>
       </c>
@@ -1925,7 +1326,7 @@
         <v>4180</v>
       </c>
       <c r="G14" s="20">
-        <f>E14*F14</f>
+        <f t="shared" si="0"/>
         <v>8360</v>
       </c>
       <c r="H14" s="19" t="s">
@@ -1939,15 +1340,15 @@
       </c>
       <c r="K14" s="7"/>
     </row>
-    <row r="15" spans="1:11" ht="15.000000">
+    <row r="15" spans="1:11" ht="13.5">
       <c r="A15" s="6"/>
       <c r="B15" s="19">
         <v>9</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="29"/>
+      <c r="D15" s="47"/>
       <c r="E15" s="22">
         <v>2</v>
       </c>
@@ -1955,7 +1356,7 @@
         <v>4180</v>
       </c>
       <c r="G15" s="20">
-        <f>E15*F15</f>
+        <f t="shared" si="0"/>
         <v>8360</v>
       </c>
       <c r="H15" s="19" t="s">
@@ -1969,15 +1370,15 @@
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="15.000000">
+    <row r="16" spans="1:11" ht="13.5">
       <c r="A16" s="6"/>
       <c r="B16" s="19">
         <v>10</v>
       </c>
-      <c r="C16" s="28" t="s">
+      <c r="C16" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="29"/>
+      <c r="D16" s="47"/>
       <c r="E16" s="22">
         <v>1</v>
       </c>
@@ -1985,7 +1386,7 @@
         <v>129800</v>
       </c>
       <c r="G16" s="20">
-        <f>E16*F16</f>
+        <f t="shared" si="0"/>
         <v>129800</v>
       </c>
       <c r="H16" s="19" t="s">
@@ -1999,15 +1400,15 @@
       </c>
       <c r="K16" s="7"/>
     </row>
-    <row r="17" spans="1:16" ht="15.000000">
+    <row r="17" spans="1:16" ht="13.5">
       <c r="A17" s="6"/>
       <c r="B17" s="19">
         <v>11</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="29"/>
+      <c r="D17" s="47"/>
       <c r="E17" s="22">
         <v>1</v>
       </c>
@@ -2015,7 +1416,7 @@
         <v>13800</v>
       </c>
       <c r="G17" s="20">
-        <f>E17*F17</f>
+        <f t="shared" si="0"/>
         <v>13800</v>
       </c>
       <c r="H17" s="19" t="s">
@@ -2029,15 +1430,15 @@
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:16" ht="15.000000">
+    <row r="18" spans="1:16" ht="13.5">
       <c r="A18" s="6"/>
       <c r="B18" s="19">
         <v>12</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="29"/>
+      <c r="D18" s="47"/>
       <c r="E18" s="22">
         <v>1</v>
       </c>
@@ -2045,7 +1446,7 @@
         <v>52800</v>
       </c>
       <c r="G18" s="20">
-        <f>E18*F18</f>
+        <f t="shared" si="0"/>
         <v>52800</v>
       </c>
       <c r="H18" s="19" t="s">
@@ -2060,15 +1461,15 @@
       <c r="K18" s="7"/>
       <c r="P18" s="13"/>
     </row>
-    <row r="19" spans="1:16" ht="15.000000">
+    <row r="19" spans="1:16" ht="13.5">
       <c r="A19" s="6"/>
       <c r="B19" s="19">
         <v>13</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="29"/>
+      <c r="D19" s="47"/>
       <c r="E19" s="22">
         <v>10</v>
       </c>
@@ -2076,7 +1477,7 @@
         <v>440</v>
       </c>
       <c r="G19" s="20">
-        <f>E19*F19</f>
+        <f t="shared" si="0"/>
         <v>4400</v>
       </c>
       <c r="H19" s="19" t="s">
@@ -2090,13 +1491,13 @@
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:16" ht="15.000000">
+    <row r="20" spans="1:16" ht="13.5">
       <c r="A20" s="6"/>
       <c r="B20" s="19">
         <v>14</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D20" s="29"/>
       <c r="E20" s="22">
@@ -2106,7 +1507,7 @@
         <v>8800</v>
       </c>
       <c r="G20" s="20">
-        <f>E20*F20</f>
+        <f t="shared" si="0"/>
         <v>17600</v>
       </c>
       <c r="H20" s="19" t="s">
@@ -2116,19 +1517,19 @@
         <v>18</v>
       </c>
       <c r="J20" s="33" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K20" s="7"/>
     </row>
-    <row r="21" spans="1:16">
+    <row r="21" spans="1:16" ht="13.5">
       <c r="A21" s="6"/>
       <c r="B21" s="19">
         <v>15</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="46" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="29"/>
+      <c r="D21" s="47"/>
       <c r="E21" s="22">
         <v>2</v>
       </c>
@@ -2136,7 +1537,7 @@
         <v>8800</v>
       </c>
       <c r="G21" s="20">
-        <f>E21*F21</f>
+        <f t="shared" si="0"/>
         <v>17600</v>
       </c>
       <c r="H21" s="19" t="s">
@@ -2150,15 +1551,15 @@
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:16" ht="15.000000">
+    <row r="22" spans="1:16" ht="13.5">
       <c r="A22" s="6"/>
       <c r="B22" s="19">
         <v>16</v>
       </c>
-      <c r="C22" s="28" t="s">
+      <c r="C22" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="29"/>
+      <c r="D22" s="47"/>
       <c r="E22" s="22">
         <v>1</v>
       </c>
@@ -2166,7 +1567,7 @@
         <v>25080</v>
       </c>
       <c r="G22" s="20">
-        <f>E22*F22</f>
+        <f t="shared" si="0"/>
         <v>25080</v>
       </c>
       <c r="H22" s="19" t="s">
@@ -2180,15 +1581,15 @@
       </c>
       <c r="K22" s="7"/>
     </row>
-    <row r="23" spans="1:16" ht="15.000000">
+    <row r="23" spans="1:16" ht="13.5">
       <c r="A23" s="6"/>
       <c r="B23" s="19">
         <v>17</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="46" t="s">
         <v>57</v>
       </c>
-      <c r="D23" s="29"/>
+      <c r="D23" s="47"/>
       <c r="E23" s="22">
         <v>1</v>
       </c>
@@ -2210,15 +1611,15 @@
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:16">
+    <row r="24" spans="1:16" ht="13.5">
       <c r="A24" s="6"/>
       <c r="B24" s="19">
         <v>18</v>
       </c>
-      <c r="C24" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="D24" s="29"/>
+      <c r="C24" s="46" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" s="47"/>
       <c r="E24" s="22">
         <v>40</v>
       </c>
@@ -2226,7 +1627,7 @@
         <v>195</v>
       </c>
       <c r="G24" s="20">
-        <f>E24*F24</f>
+        <f t="shared" ref="G24:G29" si="1">E24*F24</f>
         <v>7800</v>
       </c>
       <c r="H24" s="19" t="s">
@@ -2234,19 +1635,19 @@
       </c>
       <c r="I24" s="21"/>
       <c r="J24" s="33" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K24" s="7"/>
     </row>
-    <row r="25" spans="1:16" ht="15.000000">
+    <row r="25" spans="1:16" ht="13.5">
       <c r="A25" s="6"/>
-      <c r="B25" s="63">
+      <c r="B25" s="19">
         <v>19</v>
       </c>
-      <c r="C25" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="29"/>
+      <c r="C25" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" s="47"/>
       <c r="E25" s="22">
         <v>10</v>
       </c>
@@ -2254,7 +1655,7 @@
         <v>1430</v>
       </c>
       <c r="G25" s="20">
-        <f>E25*F25</f>
+        <f t="shared" si="1"/>
         <v>14300</v>
       </c>
       <c r="H25" s="19" t="s">
@@ -2264,19 +1665,19 @@
         <v>18</v>
       </c>
       <c r="J25" s="33" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:16" ht="15.000000">
+    <row r="26" spans="1:16" ht="13.5">
       <c r="A26" s="6"/>
       <c r="B26" s="19">
         <v>20</v>
       </c>
-      <c r="C26" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="D26" s="29"/>
+      <c r="C26" s="46" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="47"/>
       <c r="E26" s="22">
         <v>2</v>
       </c>
@@ -2284,7 +1685,7 @@
         <v>7370</v>
       </c>
       <c r="G26" s="20">
-        <f>E26*F26</f>
+        <f t="shared" si="1"/>
         <v>14740</v>
       </c>
       <c r="H26" s="19" t="s">
@@ -2294,19 +1695,19 @@
         <v>18</v>
       </c>
       <c r="J26" s="33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K26" s="7"/>
     </row>
-    <row r="27" spans="1:16" ht="15.000000">
+    <row r="27" spans="1:16" ht="13.5">
       <c r="A27" s="6"/>
-      <c r="B27" s="63">
+      <c r="B27" s="19">
         <v>21</v>
       </c>
-      <c r="C27" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="D27" s="29"/>
+      <c r="C27" s="46" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="47"/>
       <c r="E27" s="22">
         <v>1</v>
       </c>
@@ -2314,7 +1715,7 @@
         <v>13200</v>
       </c>
       <c r="G27" s="20">
-        <f>E27*F27</f>
+        <f t="shared" si="1"/>
         <v>13200</v>
       </c>
       <c r="H27" s="19" t="s">
@@ -2324,19 +1725,19 @@
         <v>18</v>
       </c>
       <c r="J27" s="33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:16" ht="15.000000">
+    <row r="28" spans="1:16" ht="13.5">
       <c r="A28" s="6"/>
-      <c r="B28" s="75">
+      <c r="B28" s="35">
         <v>22</v>
       </c>
-      <c r="C28" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="D28" s="29"/>
+      <c r="C28" s="46" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="47"/>
       <c r="E28" s="22">
         <v>4</v>
       </c>
@@ -2344,117 +1745,117 @@
         <v>48020</v>
       </c>
       <c r="G28" s="20">
-        <f>E28*F28</f>
+        <f t="shared" si="1"/>
         <v>192080</v>
       </c>
       <c r="H28" s="19" t="s">
         <v>13</v>
       </c>
       <c r="I28" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="J28" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="K28" s="7"/>
+    </row>
+    <row r="29" spans="1:16" ht="13.5">
+      <c r="A29" s="6"/>
+      <c r="B29" s="19">
+        <v>23</v>
+      </c>
+      <c r="C29" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="J28" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="K28" s="7"/>
-    </row>
-    <row r="29" spans="1:16" s="60" customFormat="1" ht="13.500000">
-      <c r="A29" s="62"/>
-      <c r="B29" s="63">
-        <v>23</v>
-      </c>
-      <c r="C29" s="64" t="s">
+      <c r="D29" s="47"/>
+      <c r="E29" s="22">
+        <v>3</v>
+      </c>
+      <c r="F29" s="20">
+        <v>1870</v>
+      </c>
+      <c r="G29" s="20">
+        <f t="shared" si="1"/>
+        <v>5610</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I29" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="J29" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="K29" s="7"/>
+    </row>
+    <row r="30" spans="1:16" ht="13.5">
+      <c r="A30" s="6"/>
+      <c r="B30" s="19">
+        <v>24</v>
+      </c>
+      <c r="C30" s="46" t="s">
         <v>76</v>
       </c>
-      <c r="D29" s="65"/>
-      <c r="E29" s="66">
+      <c r="D30" s="47"/>
+      <c r="E30" s="22">
         <v>3</v>
       </c>
-      <c r="F29" s="67">
-        <v>1870</v>
-      </c>
-      <c r="G29" s="67">
-        <f>E29*F29</f>
-        <v>5610</v>
-      </c>
-      <c r="H29" s="63" t="s">
-        <v>7</v>
-      </c>
-      <c r="I29" s="68" t="s">
-        <v>18</v>
-      </c>
-      <c r="J29" s="69" t="s">
-        <v>75</v>
-      </c>
-      <c r="K29" s="70"/>
-    </row>
-    <row r="30" spans="1:16" s="60" customFormat="1" ht="15.000000">
-      <c r="A30" s="62"/>
-      <c r="B30" s="63">
-        <v>24</v>
-      </c>
-      <c r="C30" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="D30" s="65"/>
-      <c r="E30" s="66">
-        <v>3</v>
-      </c>
-      <c r="F30" s="67">
+      <c r="F30" s="20">
         <v>8000</v>
       </c>
-      <c r="G30" s="67">
+      <c r="G30" s="20">
         <f>E30*F30+3500</f>
         <v>27500</v>
       </c>
-      <c r="H30" s="63" t="s">
+      <c r="H30" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I30" s="68" t="s">
+      <c r="I30" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="J30" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="K30" s="7"/>
+    </row>
+    <row r="31" spans="1:16" ht="13.5">
+      <c r="A31" s="6"/>
+      <c r="B31" s="19">
+        <v>25</v>
+      </c>
+      <c r="C31" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="J30" s="69" t="s">
-        <v>77</v>
-      </c>
-      <c r="K30" s="70"/>
-    </row>
-    <row r="31" spans="1:16" s="60" customFormat="1" ht="13.500000">
-      <c r="A31" s="62"/>
-      <c r="B31" s="63">
-        <v>25</v>
-      </c>
-      <c r="C31" s="64" t="s">
-        <v>81</v>
-      </c>
-      <c r="D31" s="65"/>
-      <c r="E31" s="66">
+      <c r="D31" s="47"/>
+      <c r="E31" s="22">
         <v>200</v>
       </c>
-      <c r="F31" s="67">
+      <c r="F31" s="20">
         <v>11</v>
       </c>
-      <c r="G31" s="67">
+      <c r="G31" s="20">
         <f>E31*F31</f>
         <v>2200</v>
       </c>
-      <c r="H31" s="63" t="s">
+      <c r="H31" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="I31" s="68" t="s">
+      <c r="I31" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="J31" s="69" t="s">
-        <v>80</v>
-      </c>
-      <c r="K31" s="70"/>
-    </row>
-    <row r="32" spans="1:16" ht="15.000000">
+      <c r="J31" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="K31" s="7"/>
+    </row>
+    <row r="32" spans="1:16" ht="13.5">
       <c r="A32" s="6"/>
       <c r="B32" s="19">
         <v>26</v>
       </c>
-      <c r="C32" s="28"/>
-      <c r="D32" s="29"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="47"/>
       <c r="E32" s="22"/>
       <c r="F32" s="20"/>
       <c r="G32" s="20">
@@ -2466,14 +1867,14 @@
       <c r="J32" s="21"/>
       <c r="K32" s="7"/>
     </row>
-    <row r="33" spans="1:11" ht="15.000000">
+    <row r="33" spans="1:11" ht="13.5">
       <c r="A33" s="3"/>
-      <c r="B33" s="44" t="s">
+      <c r="B33" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="45"/>
-      <c r="D33" s="45"/>
-      <c r="E33" s="46"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="50"/>
       <c r="F33" s="14" t="s">
         <v>8</v>
       </c>
@@ -2486,11 +1887,11 @@
       <c r="J33" s="17"/>
       <c r="K33" s="3"/>
     </row>
-    <row r="34" spans="1:11" ht="13.000000">
+    <row r="34" spans="1:11" ht="12.75">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="7"/>
+      <c r="C34" s="51"/>
+      <c r="D34" s="52"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -2499,15 +1900,15 @@
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
     </row>
-    <row r="35" spans="1:11" ht="13.000000">
+    <row r="35" spans="1:11" ht="12.75">
       <c r="A35" s="3"/>
       <c r="B35" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="D35" s="47"/>
+      <c r="D35" s="53"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -2516,7 +1917,7 @@
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
     </row>
-    <row r="36" spans="1:11" ht="13.000000">
+    <row r="36" spans="1:11" ht="12.75">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3" t="s">
@@ -2531,70 +1932,70 @@
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
     </row>
-    <row r="37" spans="1:11">
-      <c r="C37" s="0" t="s">
-        <v>74</v>
+    <row r="37" spans="1:11" ht="12.75">
+      <c r="C37" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H7:H26 H27 H28 H29 H30 H31">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H7:H26 H27 H28 H29 H30 H31" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"디바이스마트,쿠팡,기타"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="J8"/>
-    <hyperlink r:id="rId2" ref="J14"/>
-    <hyperlink r:id="rId3" ref="J10"/>
-    <hyperlink r:id="rId4" ref="J11"/>
-    <hyperlink r:id="rId5" ref="J9"/>
-    <hyperlink r:id="rId6" ref="J13"/>
-    <hyperlink r:id="rId7" ref="J15"/>
-    <hyperlink r:id="rId8" ref="J16"/>
-    <hyperlink r:id="rId9" ref="J12"/>
-    <hyperlink r:id="rId10" ref="J17"/>
-    <hyperlink r:id="rId11" ref="J19"/>
-    <hyperlink r:id="rId12" ref="J24"/>
-    <hyperlink r:id="rId13" ref="J29"/>
-    <hyperlink r:id="rId14" ref="J21"/>
-    <hyperlink r:id="rId15" ref="J31"/>
+    <hyperlink ref="J8" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="J14" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="J10" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="J11" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="J9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="J13" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="J15" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="J16" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="J12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="J17" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="J19" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="J24" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="J29" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="J21" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="J31" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
   </hyperlinks>
-  <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
-  <pageSetup paperSize="9" scale="59" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="59" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>